<commit_message>
daily official calendar refresh 2026-09-14 07:39:59 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6556,6 +6556,32 @@
         </is>
       </c>
       <c r="F55" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:39:59</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>31</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-15 07:19:46 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6582,6 +6582,32 @@
         </is>
       </c>
       <c r="F56" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:19:45</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="n">
+        <v>31</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-16 07:21:35 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6608,6 +6608,32 @@
         </is>
       </c>
       <c r="F57" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:21:35</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" t="n">
+        <v>31</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-17 07:17:05 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6634,6 +6634,32 @@
         </is>
       </c>
       <c r="F58" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:17:05</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" t="n">
+        <v>31</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-18 07:09:23 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6660,6 +6660,32 @@
         </is>
       </c>
       <c r="F59" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:09:22</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" t="n">
+        <v>31</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-19 07:07:07 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6686,6 +6686,32 @@
         </is>
       </c>
       <c r="F60" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-19 07:07:07</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" t="n">
+        <v>31</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-20 07:32:26 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6712,6 +6712,32 @@
         </is>
       </c>
       <c r="F61" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:32:25</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" t="n">
+        <v>31</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-21 07:43:36 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6738,6 +6738,32 @@
         </is>
       </c>
       <c r="F62" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:43:36</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" t="n">
+        <v>31</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-22 07:26:49 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6764,6 +6764,32 @@
         </is>
       </c>
       <c r="F63" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:26:49</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" t="n">
+        <v>31</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-23 07:29:09 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6790,6 +6790,32 @@
         </is>
       </c>
       <c r="F64" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:29:09</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" t="n">
+        <v>31</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-24 07:20:58 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6816,6 +6816,32 @@
         </is>
       </c>
       <c r="F65" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:20:58</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" t="n">
+        <v>31</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-25 07:14:49 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6842,6 +6842,32 @@
         </is>
       </c>
       <c r="F66" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:14:48</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" t="n">
+        <v>31</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-26 07:10:42 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6868,6 +6868,32 @@
         </is>
       </c>
       <c r="F67" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-26 07:10:41</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" t="n">
+        <v>31</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-27 07:42:32 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6894,6 +6894,32 @@
         </is>
       </c>
       <c r="F68" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-27 07:42:32</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="n">
+        <v>31</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-28 08:21:23 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6920,6 +6920,32 @@
         </is>
       </c>
       <c r="F69" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-28 08:21:23</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>31</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-29 07:59:10 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6946,6 +6946,32 @@
         </is>
       </c>
       <c r="F70" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:59:09</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>0</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="n">
+        <v>31</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-09-30 08:08:30 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6972,6 +6972,32 @@
         </is>
       </c>
       <c r="F71" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:08:30</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" t="n">
+        <v>31</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-01 08:27:01 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6998,6 +6998,32 @@
         </is>
       </c>
       <c r="F72" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-01 08:27:01</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="n">
+        <v>31</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-02 08:02:30 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7024,6 +7024,32 @@
         </is>
       </c>
       <c r="F73" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-02 08:02:30</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" t="n">
+        <v>31</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-03 07:43:58 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7050,6 +7050,32 @@
         </is>
       </c>
       <c r="F74" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-03 07:43:58</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" t="n">
+        <v>31</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-04 07:52:41 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7076,6 +7076,32 @@
         </is>
       </c>
       <c r="F75" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-04 07:52:41</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" t="n">
+        <v>31</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-05 08:31:53 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7102,6 +7102,32 @@
         </is>
       </c>
       <c r="F76" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:31:53</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" t="n">
+        <v>31</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-06 08:41:01 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7128,6 +7128,32 @@
         </is>
       </c>
       <c r="F77" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-06 08:41:01</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" t="n">
+        <v>31</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-07 08:15:29 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7154,6 +7154,32 @@
         </is>
       </c>
       <c r="F78" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-07 08:15:28</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" t="n">
+        <v>31</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-08 08:31:47 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7180,6 +7180,32 @@
         </is>
       </c>
       <c r="F79" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:31:47</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" t="n">
+        <v>31</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-09 08:35:20 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7206,6 +7206,32 @@
         </is>
       </c>
       <c r="F80" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-09 08:35:20</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" t="n">
+        <v>31</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-10 08:12:08 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7232,6 +7232,32 @@
         </is>
       </c>
       <c r="F81" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-10 08:12:08</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" t="n">
+        <v>31</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-11 08:23:45 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7258,6 +7258,32 @@
         </is>
       </c>
       <c r="F82" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-11 08:23:44</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" t="n">
+        <v>31</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-12 08:46:30 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7284,6 +7284,32 @@
         </is>
       </c>
       <c r="F83" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-12 08:46:30</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" t="n">
+        <v>31</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-13 09:04:09 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7310,6 +7310,32 @@
         </is>
       </c>
       <c r="F84" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-13 09:04:09</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" t="n">
+        <v>31</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-14 07:13:47 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7336,6 +7336,32 @@
         </is>
       </c>
       <c r="F85" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:13:47</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" t="n">
+        <v>31</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-15 07:05:22 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7362,6 +7362,32 @@
         </is>
       </c>
       <c r="F86" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:05:22</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="n">
+        <v>31</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-16 06:48:59 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7388,6 +7388,32 @@
         </is>
       </c>
       <c r="F87" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-16 06:48:59</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" t="n">
+        <v>31</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-17 06:41:28 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7414,6 +7414,32 @@
         </is>
       </c>
       <c r="F88" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-17 06:41:27</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" t="n">
+        <v>31</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-18 07:02:35 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7440,6 +7440,32 @@
         </is>
       </c>
       <c r="F89" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-18 07:02:35</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" t="n">
+        <v>31</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-19 07:25:52 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7466,6 +7466,32 @@
         </is>
       </c>
       <c r="F90" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:25:52</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="n">
+        <v>31</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-20 07:16:16 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7492,6 +7492,32 @@
         </is>
       </c>
       <c r="F91" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:16:16</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" t="n">
+        <v>31</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-21 07:11:29 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7518,6 +7518,32 @@
         </is>
       </c>
       <c r="F92" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:11:28</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" t="n">
+        <v>31</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-22 07:13:59 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7544,6 +7544,32 @@
         </is>
       </c>
       <c r="F93" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:13:59</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" t="n">
+        <v>31</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-23 07:05:41 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7570,6 +7570,32 @@
         </is>
       </c>
       <c r="F94" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-23 07:05:41</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" t="n">
+        <v>31</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-24 06:57:52 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7596,6 +7596,32 @@
         </is>
       </c>
       <c r="F95" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-24 06:57:51</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" t="n">
+        <v>31</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-25 07:21:31 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7622,6 +7622,32 @@
         </is>
       </c>
       <c r="F96" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:21:31</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" t="n">
+        <v>31</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-26 07:30:38 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7648,6 +7648,32 @@
         </is>
       </c>
       <c r="F97" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:30:37</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" t="n">
+        <v>31</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-27 07:26:25 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7674,6 +7674,32 @@
         </is>
       </c>
       <c r="F98" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:26:25</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" t="n">
+        <v>31</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-28 08:00:30 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7700,6 +7700,32 @@
         </is>
       </c>
       <c r="F99" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-28 08:00:30</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" t="n">
+        <v>31</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-29 08:09:11 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7726,6 +7726,32 @@
         </is>
       </c>
       <c r="F100" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-29 08:09:11</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" t="n">
+        <v>31</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-30 08:11:56 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7752,6 +7752,32 @@
         </is>
       </c>
       <c r="F101" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-10-30 08:11:56</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>0</v>
+      </c>
+      <c r="C102" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" t="n">
+        <v>31</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>

<commit_message>
daily official calendar refresh 2026-10-31 08:05:24 updated=0 candidates=0
</commit_message>
<xml_diff>
--- a/data/holiday_student_analysis.xlsx
+++ b/data/holiday_student_analysis.xlsx
@@ -5122,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7778,6 +7778,32 @@
         </is>
       </c>
       <c r="F102" t="inlineStr">
+        <is>
+          <t>准备生成看板并同步 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-31 08:05:24</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" t="n">
+        <v>31</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
         <is>
           <t>准备生成看板并同步 GitHub</t>
         </is>

</xml_diff>